<commit_message>
updated SAV analysis 04-20-2026
</commit_message>
<xml_diff>
--- a/SAV/output/website/SAV_BBpct_LMEresults_All.xlsx
+++ b/SAV/output/website/SAV_BBpct_LMEresults_All.xlsx
@@ -191,7 +191,7 @@
     <t xml:space="preserve">965, 4018, 4049</t>
   </si>
   <si>
-    <t xml:space="preserve">Miami-Dade County DERM Benthic Habitat Monitoring Program, North Biscayne Bay Seagrass Loss Monitoring Program, South Florida Seagrass Fish and Invertebrate Assessment Network, The South Florida Fisheries Habitat Assessment Program (FHAP)</t>
+    <t xml:space="preserve">Miami-Dade County DERM Benthic Habitat Monitoring Program, North Biscayne Bay Seagrass Monitoring Program, South Florida Seagrass Fish and Invertebrate Assessment Network, The South Florida Fisheries Habitat Assessment Program (FHAP)</t>
   </si>
   <si>
     <t xml:space="preserve">965, 4018, 4049, 5027</t>
@@ -827,13 +827,13 @@
         <v>1</v>
       </c>
       <c r="M2" t="n">
-        <v>79.4029214173515</v>
+        <v>79.4024458379973</v>
       </c>
       <c r="N2" t="n">
-        <v>-2.35626636964849</v>
+        <v>-2.3562408050717</v>
       </c>
       <c r="O2" t="n">
-        <v>0.0273449574529121</v>
+        <v>0.0273462910086319</v>
       </c>
       <c r="P2" t="s">
         <v>21</v>
@@ -877,13 +877,13 @@
         <v>1</v>
       </c>
       <c r="M3" t="n">
-        <v>29.7876434404689</v>
+        <v>29.7876385227131</v>
       </c>
       <c r="N3" t="n">
-        <v>-0.499367096337099</v>
+        <v>-0.499366822442305</v>
       </c>
       <c r="O3" t="n">
-        <v>0.47169123539315</v>
+        <v>0.471691483034255</v>
       </c>
       <c r="P3" t="s">
         <v>23</v>
@@ -1059,13 +1059,13 @@
         <v>1</v>
       </c>
       <c r="M7" t="n">
-        <v>47.8583554328725</v>
+        <v>47.8583559827204</v>
       </c>
       <c r="N7" t="n">
-        <v>-1.22814508288897</v>
+        <v>-1.22814510144716</v>
       </c>
       <c r="O7" t="n">
-        <v>0.0253567863646845</v>
+        <v>0.0253567825587495</v>
       </c>
       <c r="P7" t="s">
         <v>21</v>
@@ -1109,13 +1109,13 @@
         <v>1</v>
       </c>
       <c r="M8" t="n">
-        <v>30.9690324948559</v>
+        <v>30.9690281919503</v>
       </c>
       <c r="N8" t="n">
-        <v>-0.453089171674389</v>
+        <v>-0.453089114504738</v>
       </c>
       <c r="O8" t="n">
-        <v>0.377857977930008</v>
+        <v>0.37785757960882</v>
       </c>
       <c r="P8" t="s">
         <v>23</v>
@@ -1159,13 +1159,13 @@
         <v>1</v>
       </c>
       <c r="M9" t="n">
-        <v>84.8219702012535</v>
+        <v>84.8219501837185</v>
       </c>
       <c r="N9" t="n">
-        <v>-2.63096007154072</v>
+        <v>-2.63095713712759</v>
       </c>
       <c r="O9" t="n">
-        <v>0.00143449561043848</v>
+        <v>0.00143440332984336</v>
       </c>
       <c r="P9" t="s">
         <v>21</v>
@@ -1209,13 +1209,13 @@
         <v>1</v>
       </c>
       <c r="M10" t="n">
-        <v>31.689931606138</v>
+        <v>31.6899376314409</v>
       </c>
       <c r="N10" t="n">
-        <v>0.916393272319195</v>
+        <v>0.916393045143222</v>
       </c>
       <c r="O10" t="n">
-        <v>0.487611162523752</v>
+        <v>0.487611201074338</v>
       </c>
       <c r="P10" t="s">
         <v>23</v>
@@ -1347,13 +1347,13 @@
         <v>1</v>
       </c>
       <c r="M13" t="n">
-        <v>60.3078035654648</v>
+        <v>60.3086992409572</v>
       </c>
       <c r="N13" t="n">
-        <v>-1.83626458333325</v>
+        <v>-1.83629600396035</v>
       </c>
       <c r="O13" t="n">
-        <v>0.0314669515239364</v>
+        <v>0.0314622501331645</v>
       </c>
       <c r="P13" t="s">
         <v>21</v>
@@ -1397,13 +1397,13 @@
         <v>1</v>
       </c>
       <c r="M14" t="n">
-        <v>42.9808649251357</v>
+        <v>42.9808695316888</v>
       </c>
       <c r="N14" t="n">
-        <v>-0.244491943134917</v>
+        <v>-0.244492117921787</v>
       </c>
       <c r="O14" t="n">
-        <v>0.726844670485489</v>
+        <v>0.726844468394392</v>
       </c>
       <c r="P14" t="s">
         <v>23</v>
@@ -1648,28 +1648,28 @@
         <v>43</v>
       </c>
       <c r="H20" t="n">
-        <v>5015</v>
+        <v>5129</v>
       </c>
       <c r="I20" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J20" t="n">
         <v>1997</v>
       </c>
       <c r="K20" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L20" t="b">
         <v>1</v>
       </c>
       <c r="M20" t="n">
-        <v>33.9007874331586</v>
+        <v>32.7066091430685</v>
       </c>
       <c r="N20" t="n">
-        <v>-1.35742555341704</v>
+        <v>-1.27421024612962</v>
       </c>
       <c r="O20" t="n">
-        <v>0.000000000000000000000000203377469239067</v>
+        <v>0.00000000000000000000000000234034760816071</v>
       </c>
       <c r="P20" t="s">
         <v>21</v>
@@ -1698,31 +1698,31 @@
         <v>43</v>
       </c>
       <c r="H21" t="n">
-        <v>15099</v>
+        <v>15441</v>
       </c>
       <c r="I21" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J21" t="n">
         <v>1997</v>
       </c>
       <c r="K21" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L21" t="b">
         <v>1</v>
       </c>
       <c r="M21" t="n">
-        <v>0.586438098835243</v>
+        <v>0.499717286812712</v>
       </c>
       <c r="N21" t="n">
-        <v>-0.0187455406333436</v>
+        <v>-0.0130908444524584</v>
       </c>
       <c r="O21" t="n">
-        <v>0.00260339690177092</v>
+        <v>0.1417157133767</v>
       </c>
       <c r="P21" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="22">
@@ -1748,28 +1748,28 @@
         <v>43</v>
       </c>
       <c r="H22" t="n">
-        <v>5017</v>
+        <v>5131</v>
       </c>
       <c r="I22" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J22" t="n">
         <v>1997</v>
       </c>
       <c r="K22" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L22" t="b">
         <v>1</v>
       </c>
       <c r="M22" t="n">
-        <v>8.1349572946358</v>
+        <v>7.79828345677389</v>
       </c>
       <c r="N22" t="n">
-        <v>-0.368128240338782</v>
+        <v>-0.344328370167375</v>
       </c>
       <c r="O22" t="n">
-        <v>0.000220172022349172</v>
+        <v>0.000230385165200919</v>
       </c>
       <c r="P22" t="s">
         <v>21</v>
@@ -1798,28 +1798,28 @@
         <v>43</v>
       </c>
       <c r="H23" t="n">
-        <v>5033</v>
+        <v>5147</v>
       </c>
       <c r="I23" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J23" t="n">
         <v>1997</v>
       </c>
       <c r="K23" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L23" t="b">
         <v>1</v>
       </c>
       <c r="M23" t="n">
-        <v>0.0920067229315442</v>
+        <v>0.0924090068810235</v>
       </c>
       <c r="N23" t="n">
-        <v>-0.00281889011236782</v>
+        <v>-0.00286056085647991</v>
       </c>
       <c r="O23" t="n">
-        <v>0.0740554281068865</v>
+        <v>0.0682854623978636</v>
       </c>
       <c r="P23" t="s">
         <v>23</v>
@@ -1848,16 +1848,16 @@
         <v>43</v>
       </c>
       <c r="H24" t="n">
-        <v>5033</v>
+        <v>5147</v>
       </c>
       <c r="I24" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J24" t="n">
         <v>1997</v>
       </c>
       <c r="K24" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L24" t="b">
         <v>1</v>
@@ -1892,28 +1892,28 @@
         <v>43</v>
       </c>
       <c r="H25" t="n">
-        <v>5268</v>
+        <v>5382</v>
       </c>
       <c r="I25" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="J25" t="n">
         <v>1994</v>
       </c>
       <c r="K25" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L25" t="b">
         <v>1</v>
       </c>
       <c r="M25" t="n">
-        <v>40.2866137603621</v>
+        <v>39.0719765042805</v>
       </c>
       <c r="N25" t="n">
-        <v>-1.61058688172235</v>
+        <v>-1.51988946018712</v>
       </c>
       <c r="O25" t="n">
-        <v>0.000000000000000000722113633213353</v>
+        <v>0.00000000000000000016644362385066</v>
       </c>
       <c r="P25" t="s">
         <v>21</v>
@@ -1997,13 +1997,13 @@
         <v>1</v>
       </c>
       <c r="M27" t="n">
-        <v>5.45391072011971</v>
+        <v>5.4539122005051</v>
       </c>
       <c r="N27" t="n">
-        <v>0.812732977917008</v>
+        <v>0.812732920657474</v>
       </c>
       <c r="O27" t="n">
-        <v>0.000000874242615872593</v>
+        <v>0.000000874243938426819</v>
       </c>
       <c r="P27" t="s">
         <v>50</v>
@@ -2047,13 +2047,13 @@
         <v>1</v>
       </c>
       <c r="M28" t="n">
-        <v>24.8297466095871</v>
+        <v>24.8297465486173</v>
       </c>
       <c r="N28" t="n">
-        <v>-0.431455086397473</v>
+        <v>-0.431455084497684</v>
       </c>
       <c r="O28" t="n">
-        <v>0.000128012089267812</v>
+        <v>0.000128012104588442</v>
       </c>
       <c r="P28" t="s">
         <v>21</v>
@@ -2097,13 +2097,13 @@
         <v>1</v>
       </c>
       <c r="M29" t="n">
-        <v>18.5527893672857</v>
+        <v>18.552789337222</v>
       </c>
       <c r="N29" t="n">
-        <v>-0.134772662261152</v>
+        <v>-0.134772661241874</v>
       </c>
       <c r="O29" t="n">
-        <v>0.308991267684262</v>
+        <v>0.308991284377083</v>
       </c>
       <c r="P29" t="s">
         <v>23</v>
@@ -2191,13 +2191,13 @@
         <v>1</v>
       </c>
       <c r="M31" t="n">
-        <v>25.9396036229984</v>
+        <v>25.9396728282327</v>
       </c>
       <c r="N31" t="n">
-        <v>-0.27930890670535</v>
+        <v>-0.279328433842235</v>
       </c>
       <c r="O31" t="n">
-        <v>0.598258418024884</v>
+        <v>0.598233856707755</v>
       </c>
       <c r="P31" t="s">
         <v>23</v>
@@ -2241,13 +2241,13 @@
         <v>1</v>
       </c>
       <c r="M32" t="n">
-        <v>35.9453958070078</v>
+        <v>35.9453957791293</v>
       </c>
       <c r="N32" t="n">
-        <v>-0.427177117773613</v>
+        <v>-0.42717713570092</v>
       </c>
       <c r="O32" t="n">
-        <v>0.000053598015625151</v>
+        <v>0.0000535982091523411</v>
       </c>
       <c r="P32" t="s">
         <v>21</v>
@@ -2291,13 +2291,13 @@
         <v>1</v>
       </c>
       <c r="M33" t="n">
-        <v>42.516006174884</v>
+        <v>42.5154354067174</v>
       </c>
       <c r="N33" t="n">
-        <v>-0.481511166139247</v>
+        <v>-0.481472297581496</v>
       </c>
       <c r="O33" t="n">
-        <v>0.000000000600899754674316</v>
+        <v>0.000000000604370552252266</v>
       </c>
       <c r="P33" t="s">
         <v>21</v>
@@ -2341,13 +2341,13 @@
         <v>1</v>
       </c>
       <c r="M34" t="n">
-        <v>-0.0338584136116649</v>
+        <v>-0.0338584442431049</v>
       </c>
       <c r="N34" t="n">
-        <v>0.00963406012485885</v>
+        <v>0.0096340617960582</v>
       </c>
       <c r="O34" t="n">
-        <v>0.102881512925586</v>
+        <v>0.102881423110622</v>
       </c>
       <c r="P34" t="s">
         <v>23</v>
@@ -2376,7 +2376,7 @@
         <v>58</v>
       </c>
       <c r="H35" t="n">
-        <v>11249</v>
+        <v>11252</v>
       </c>
       <c r="I35" t="n">
         <v>26</v>
@@ -2391,13 +2391,13 @@
         <v>1</v>
       </c>
       <c r="M35" t="n">
-        <v>10.7300595601416</v>
+        <v>10.7299717287469</v>
       </c>
       <c r="N35" t="n">
-        <v>-0.313698497351088</v>
+        <v>-0.313686425316573</v>
       </c>
       <c r="O35" t="n">
-        <v>0.000000497673940350208</v>
+        <v>0.000000494818421991087</v>
       </c>
       <c r="P35" t="s">
         <v>21</v>
@@ -2426,7 +2426,7 @@
         <v>60</v>
       </c>
       <c r="H36" t="n">
-        <v>13865</v>
+        <v>13868</v>
       </c>
       <c r="I36" t="n">
         <v>26</v>
@@ -2441,13 +2441,13 @@
         <v>1</v>
       </c>
       <c r="M36" t="n">
-        <v>8.20628315088408</v>
+        <v>8.20630451675424</v>
       </c>
       <c r="N36" t="n">
-        <v>-0.23154704325086</v>
+        <v>-0.23154800185622</v>
       </c>
       <c r="O36" t="n">
-        <v>0.00000613290236282766</v>
+        <v>0.00000610770243154178</v>
       </c>
       <c r="P36" t="s">
         <v>21</v>
@@ -2476,7 +2476,7 @@
         <v>60</v>
       </c>
       <c r="H37" t="n">
-        <v>40514</v>
+        <v>40526</v>
       </c>
       <c r="I37" t="n">
         <v>25</v>
@@ -2491,13 +2491,13 @@
         <v>1</v>
       </c>
       <c r="M37" t="n">
-        <v>0.668606372700147</v>
+        <v>0.668645792189909</v>
       </c>
       <c r="N37" t="n">
-        <v>-0.0227167001769804</v>
+        <v>-0.022717678236175</v>
       </c>
       <c r="O37" t="n">
-        <v>0.00941316007048729</v>
+        <v>0.00940484396388284</v>
       </c>
       <c r="P37" t="s">
         <v>21</v>
@@ -2526,7 +2526,7 @@
         <v>58</v>
       </c>
       <c r="H38" t="n">
-        <v>9335</v>
+        <v>9338</v>
       </c>
       <c r="I38" t="n">
         <v>20</v>
@@ -2570,7 +2570,7 @@
         <v>60</v>
       </c>
       <c r="H39" t="n">
-        <v>13788</v>
+        <v>13791</v>
       </c>
       <c r="I39" t="n">
         <v>26</v>
@@ -2585,13 +2585,13 @@
         <v>1</v>
       </c>
       <c r="M39" t="n">
-        <v>14.7507003028008</v>
+        <v>14.7500249367134</v>
       </c>
       <c r="N39" t="n">
-        <v>-0.370286460260618</v>
+        <v>-0.370260581585335</v>
       </c>
       <c r="O39" t="n">
-        <v>0.000282124323879578</v>
+        <v>0.000281397786247974</v>
       </c>
       <c r="P39" t="s">
         <v>21</v>
@@ -2620,7 +2620,7 @@
         <v>60</v>
       </c>
       <c r="H40" t="n">
-        <v>14080</v>
+        <v>14083</v>
       </c>
       <c r="I40" t="n">
         <v>26</v>
@@ -2635,13 +2635,13 @@
         <v>1</v>
       </c>
       <c r="M40" t="n">
-        <v>45.0504478399706</v>
+        <v>44.9650111183382</v>
       </c>
       <c r="N40" t="n">
-        <v>-1.37948295410189</v>
+        <v>-1.37407678080075</v>
       </c>
       <c r="O40" t="n">
-        <v>0.000000000000000000000000000230874001990556</v>
+        <v>0.000000000000000000000000000125679599318174</v>
       </c>
       <c r="P40" t="s">
         <v>21</v>
@@ -2670,7 +2670,7 @@
         <v>58</v>
       </c>
       <c r="H41" t="n">
-        <v>9399</v>
+        <v>9402</v>
       </c>
       <c r="I41" t="n">
         <v>26</v>
@@ -2685,13 +2685,13 @@
         <v>1</v>
       </c>
       <c r="M41" t="n">
-        <v>51.3012406323683</v>
+        <v>51.2374696438551</v>
       </c>
       <c r="N41" t="n">
-        <v>-0.210720901565839</v>
+        <v>-0.206500310474665</v>
       </c>
       <c r="O41" t="n">
-        <v>0.246747964706292</v>
+        <v>0.256494287264958</v>
       </c>
       <c r="P41" t="s">
         <v>23</v>
@@ -2720,7 +2720,7 @@
         <v>60</v>
       </c>
       <c r="H42" t="n">
-        <v>11998</v>
+        <v>12001</v>
       </c>
       <c r="I42" t="n">
         <v>20</v>
@@ -2735,13 +2735,13 @@
         <v>1</v>
       </c>
       <c r="M42" t="n">
-        <v>17.1668352676616</v>
+        <v>17.1355555254218</v>
       </c>
       <c r="N42" t="n">
-        <v>0.606021674072554</v>
+        <v>0.607696990107161</v>
       </c>
       <c r="O42" t="n">
-        <v>0.00127316757816461</v>
+        <v>0.00122802477495601</v>
       </c>
       <c r="P42" t="s">
         <v>50</v>
@@ -2829,13 +2829,13 @@
         <v>1</v>
       </c>
       <c r="M44" t="n">
-        <v>47.9776204495857</v>
+        <v>47.9776204495858</v>
       </c>
       <c r="N44" t="n">
-        <v>-0.198288963007622</v>
+        <v>-0.198288963007626</v>
       </c>
       <c r="O44" t="n">
-        <v>0.377609133307048</v>
+        <v>0.377609133307038</v>
       </c>
       <c r="P44" t="s">
         <v>23</v>
@@ -2967,13 +2967,13 @@
         <v>1</v>
       </c>
       <c r="M47" t="n">
-        <v>52.3263057424217</v>
+        <v>52.3267182771389</v>
       </c>
       <c r="N47" t="n">
-        <v>-0.496445020780152</v>
+        <v>-0.496461552365028</v>
       </c>
       <c r="O47" t="n">
-        <v>0.0492309598769332</v>
+        <v>0.0491914585084037</v>
       </c>
       <c r="P47" t="s">
         <v>21</v>
@@ -3105,13 +3105,13 @@
         <v>1</v>
       </c>
       <c r="M50" t="n">
-        <v>-11.4840673786696</v>
+        <v>-11.4840654985292</v>
       </c>
       <c r="N50" t="n">
-        <v>1.24661540748319</v>
+        <v>1.24661532602356</v>
       </c>
       <c r="O50" t="n">
-        <v>0.0166233333045051</v>
+        <v>0.0166233464754912</v>
       </c>
       <c r="P50" t="s">
         <v>50</v>
@@ -3155,13 +3155,13 @@
         <v>1</v>
       </c>
       <c r="M51" t="n">
-        <v>21.9819548961927</v>
+        <v>21.9823058362862</v>
       </c>
       <c r="N51" t="n">
-        <v>-0.330012373168787</v>
+        <v>-0.330017781273232</v>
       </c>
       <c r="O51" t="n">
-        <v>0.348782449920717</v>
+        <v>0.348779258545112</v>
       </c>
       <c r="P51" t="s">
         <v>23</v>
@@ -3249,13 +3249,13 @@
         <v>1</v>
       </c>
       <c r="M53" t="n">
-        <v>31.3222862611413</v>
+        <v>31.3183097469319</v>
       </c>
       <c r="N53" t="n">
-        <v>-0.165135704523702</v>
+        <v>-0.164982613440194</v>
       </c>
       <c r="O53" t="n">
-        <v>0.831128064926257</v>
+        <v>0.83124841287508</v>
       </c>
       <c r="P53" t="s">
         <v>23</v>
@@ -3299,13 +3299,13 @@
         <v>1</v>
       </c>
       <c r="M54" t="n">
-        <v>24.5778014751751</v>
+        <v>24.5774894460146</v>
       </c>
       <c r="N54" t="n">
-        <v>0.218495167677927</v>
+        <v>0.21849050167077</v>
       </c>
       <c r="O54" t="n">
-        <v>0.483422207860359</v>
+        <v>0.483437203484199</v>
       </c>
       <c r="P54" t="s">
         <v>23</v>
@@ -3349,13 +3349,13 @@
         <v>1</v>
       </c>
       <c r="M55" t="n">
-        <v>31.2028300204007</v>
+        <v>31.2028301375394</v>
       </c>
       <c r="N55" t="n">
-        <v>-0.394610085552156</v>
+        <v>-0.394610092902706</v>
       </c>
       <c r="O55" t="n">
-        <v>0.320530875879872</v>
+        <v>0.320530874580492</v>
       </c>
       <c r="P55" t="s">
         <v>23</v>
@@ -3487,13 +3487,13 @@
         <v>1</v>
       </c>
       <c r="M58" t="n">
-        <v>19.2210209388705</v>
+        <v>19.2210209918651</v>
       </c>
       <c r="N58" t="n">
-        <v>0.529458795534344</v>
+        <v>0.529458794026777</v>
       </c>
       <c r="O58" t="n">
-        <v>0.0159141933378494</v>
+        <v>0.0159141893678147</v>
       </c>
       <c r="P58" t="s">
         <v>50</v>
@@ -3581,13 +3581,13 @@
         <v>1</v>
       </c>
       <c r="M60" t="n">
-        <v>35.7777232495791</v>
+        <v>35.7777215434534</v>
       </c>
       <c r="N60" t="n">
-        <v>0.825668232311731</v>
+        <v>0.825668344603955</v>
       </c>
       <c r="O60" t="n">
-        <v>0.0760965115153528</v>
+        <v>0.0760969879640776</v>
       </c>
       <c r="P60" t="s">
         <v>23</v>
@@ -3631,13 +3631,13 @@
         <v>1</v>
       </c>
       <c r="M61" t="n">
-        <v>16.2416050985637</v>
+        <v>16.2416047164727</v>
       </c>
       <c r="N61" t="n">
-        <v>0.175117442874633</v>
+        <v>0.175117461352373</v>
       </c>
       <c r="O61" t="n">
-        <v>0.42480740143852</v>
+        <v>0.424807329805699</v>
       </c>
       <c r="P61" t="s">
         <v>23</v>
@@ -3725,13 +3725,13 @@
         <v>1</v>
       </c>
       <c r="M63" t="n">
-        <v>8.13470865386613</v>
+        <v>8.13470493366117</v>
       </c>
       <c r="N63" t="n">
-        <v>-0.201985152177262</v>
+        <v>-0.201984889529685</v>
       </c>
       <c r="O63" t="n">
-        <v>0.386178912889689</v>
+        <v>0.386180086961865</v>
       </c>
       <c r="P63" t="s">
         <v>23</v>
@@ -3775,13 +3775,13 @@
         <v>1</v>
       </c>
       <c r="M64" t="n">
-        <v>20.0363360971138</v>
+        <v>20.0363360880779</v>
       </c>
       <c r="N64" t="n">
-        <v>-0.287623337709177</v>
+        <v>-0.287623336006212</v>
       </c>
       <c r="O64" t="n">
-        <v>0.37852297795719</v>
+        <v>0.378522951480508</v>
       </c>
       <c r="P64" t="s">
         <v>23</v>
@@ -3825,13 +3825,13 @@
         <v>1</v>
       </c>
       <c r="M65" t="n">
-        <v>37.073941318164</v>
+        <v>37.0739399502456</v>
       </c>
       <c r="N65" t="n">
-        <v>-0.830567769864988</v>
+        <v>-0.830567730486169</v>
       </c>
       <c r="O65" t="n">
-        <v>0.00105845486851883</v>
+        <v>0.0010585081754943</v>
       </c>
       <c r="P65" t="s">
         <v>21</v>
@@ -3875,13 +3875,13 @@
         <v>1</v>
       </c>
       <c r="M66" t="n">
-        <v>18.8993364838794</v>
+        <v>18.8993364617153</v>
       </c>
       <c r="N66" t="n">
-        <v>-0.0551538065310624</v>
+        <v>-0.0551538224617119</v>
       </c>
       <c r="O66" t="n">
-        <v>0.922197373226081</v>
+        <v>0.92219735068256</v>
       </c>
       <c r="P66" t="s">
         <v>23</v>
@@ -4013,13 +4013,13 @@
         <v>1</v>
       </c>
       <c r="M69" t="n">
-        <v>26.9390954778279</v>
+        <v>26.9390749103907</v>
       </c>
       <c r="N69" t="n">
-        <v>-0.972095996812152</v>
+        <v>-0.972109067084369</v>
       </c>
       <c r="O69" t="n">
-        <v>0.351760435718147</v>
+        <v>0.351749557583809</v>
       </c>
       <c r="P69" t="s">
         <v>23</v>
@@ -4063,13 +4063,13 @@
         <v>1</v>
       </c>
       <c r="M70" t="n">
-        <v>22.4462541270106</v>
+        <v>22.4462540765769</v>
       </c>
       <c r="N70" t="n">
-        <v>-0.47904710977692</v>
+        <v>-0.479047107062301</v>
       </c>
       <c r="O70" t="n">
-        <v>0.0101183615661718</v>
+        <v>0.0101183628293739</v>
       </c>
       <c r="P70" t="s">
         <v>21</v>
@@ -4113,13 +4113,13 @@
         <v>1</v>
       </c>
       <c r="M71" t="n">
-        <v>47.6649674238452</v>
+        <v>47.6649674238473</v>
       </c>
       <c r="N71" t="n">
-        <v>-1.27036875345826</v>
+        <v>-1.27036875345833</v>
       </c>
       <c r="O71" t="n">
-        <v>0.0235055099480932</v>
+        <v>0.0235055099480849</v>
       </c>
       <c r="P71" t="s">
         <v>21</v>
@@ -4192,28 +4192,28 @@
         <v>56</v>
       </c>
       <c r="H73" t="n">
-        <v>9132</v>
+        <v>9660</v>
       </c>
       <c r="I73" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J73" t="n">
         <v>2008</v>
       </c>
       <c r="K73" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L73" t="b">
         <v>1</v>
       </c>
       <c r="M73" t="n">
-        <v>0.0758368299035063</v>
+        <v>0.0741863485323382</v>
       </c>
       <c r="N73" t="n">
-        <v>-0.00252875986567735</v>
+        <v>-0.00244914775312295</v>
       </c>
       <c r="O73" t="n">
-        <v>0.21189295104168</v>
+        <v>0.196740148903206</v>
       </c>
       <c r="P73" t="s">
         <v>23</v>
@@ -4242,28 +4242,28 @@
         <v>58</v>
       </c>
       <c r="H74" t="n">
-        <v>17509</v>
+        <v>18037</v>
       </c>
       <c r="I74" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="J74" t="n">
         <v>1999</v>
       </c>
       <c r="K74" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L74" t="b">
         <v>1</v>
       </c>
       <c r="M74" t="n">
-        <v>9.03257305752796</v>
+        <v>8.74319566013521</v>
       </c>
       <c r="N74" t="n">
-        <v>-0.225030998869794</v>
+        <v>-0.20777732678382</v>
       </c>
       <c r="O74" t="n">
-        <v>0.0000182151319884356</v>
+        <v>0.0000785983600721293</v>
       </c>
       <c r="P74" t="s">
         <v>21</v>
@@ -4292,28 +4292,28 @@
         <v>77</v>
       </c>
       <c r="H75" t="n">
-        <v>18961</v>
+        <v>19551</v>
       </c>
       <c r="I75" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="J75" t="n">
         <v>1996</v>
       </c>
       <c r="K75" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L75" t="b">
         <v>1</v>
       </c>
       <c r="M75" t="n">
-        <v>6.73486166531502</v>
+        <v>6.65893014025401</v>
       </c>
       <c r="N75" t="n">
-        <v>-0.249327439209218</v>
+        <v>-0.244005551617337</v>
       </c>
       <c r="O75" t="n">
-        <v>0.000222134049987985</v>
+        <v>0.000291230507719468</v>
       </c>
       <c r="P75" t="s">
         <v>21</v>
@@ -4342,28 +4342,28 @@
         <v>79</v>
       </c>
       <c r="H76" t="n">
-        <v>46762</v>
+        <v>47846</v>
       </c>
       <c r="I76" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J76" t="n">
         <v>2005</v>
       </c>
       <c r="K76" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L76" t="b">
         <v>1</v>
       </c>
       <c r="M76" t="n">
-        <v>0.0759972082175504</v>
+        <v>0.0693824791412447</v>
       </c>
       <c r="N76" t="n">
-        <v>-0.00236205422017377</v>
+        <v>-0.00186620090774331</v>
       </c>
       <c r="O76" t="n">
-        <v>0.303057711180532</v>
+        <v>0.413500371689689</v>
       </c>
       <c r="P76" t="s">
         <v>23</v>
@@ -4392,28 +4392,28 @@
         <v>81</v>
       </c>
       <c r="H77" t="n">
-        <v>17002</v>
+        <v>17558</v>
       </c>
       <c r="I77" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J77" t="n">
         <v>2005</v>
       </c>
       <c r="K77" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L77" t="b">
         <v>1</v>
       </c>
       <c r="M77" t="n">
-        <v>-0.037620182191274</v>
+        <v>-0.0286063078687182</v>
       </c>
       <c r="N77" t="n">
-        <v>0.00276837307072622</v>
+        <v>0.00220465781341062</v>
       </c>
       <c r="O77" t="n">
-        <v>0.104988262573557</v>
+        <v>0.127260017280868</v>
       </c>
       <c r="P77" t="s">
         <v>23</v>
@@ -4442,28 +4442,28 @@
         <v>77</v>
       </c>
       <c r="H78" t="n">
-        <v>18880</v>
+        <v>19436</v>
       </c>
       <c r="I78" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="J78" t="n">
         <v>1996</v>
       </c>
       <c r="K78" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L78" t="b">
         <v>1</v>
       </c>
       <c r="M78" t="n">
-        <v>4.88761818989823</v>
+        <v>4.94124465717422</v>
       </c>
       <c r="N78" t="n">
-        <v>-0.106401736366778</v>
+        <v>-0.107991097626809</v>
       </c>
       <c r="O78" t="n">
-        <v>0.0205244100822212</v>
+        <v>0.0175021586314602</v>
       </c>
       <c r="P78" t="s">
         <v>21</v>
@@ -4492,28 +4492,28 @@
         <v>77</v>
       </c>
       <c r="H79" t="n">
-        <v>19201</v>
+        <v>19879</v>
       </c>
       <c r="I79" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="J79" t="n">
         <v>1996</v>
       </c>
       <c r="K79" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L79" t="b">
         <v>1</v>
       </c>
       <c r="M79" t="n">
-        <v>43.3088390618793</v>
+        <v>42.2873517846192</v>
       </c>
       <c r="N79" t="n">
-        <v>-1.42664895537423</v>
+        <v>-1.38206015255954</v>
       </c>
       <c r="O79" t="n">
-        <v>0.00000000000000000000000000000198475441221113</v>
+        <v>0.000000000000000000000000000505749538387561</v>
       </c>
       <c r="P79" t="s">
         <v>21</v>
@@ -4542,28 +4542,28 @@
         <v>58</v>
       </c>
       <c r="H80" t="n">
-        <v>16233</v>
+        <v>16804</v>
       </c>
       <c r="I80" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="J80" t="n">
         <v>1999</v>
       </c>
       <c r="K80" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L80" t="b">
         <v>1</v>
       </c>
       <c r="M80" t="n">
-        <v>31.6516899923504</v>
+        <v>31.2798285343373</v>
       </c>
       <c r="N80" t="n">
-        <v>0.215667371185139</v>
+        <v>0.237657083252429</v>
       </c>
       <c r="O80" t="n">
-        <v>0.164546093099561</v>
+        <v>0.116657820450709</v>
       </c>
       <c r="P80" t="s">
         <v>23</v>
@@ -4592,28 +4592,28 @@
         <v>79</v>
       </c>
       <c r="H81" t="n">
-        <v>15943</v>
+        <v>16627</v>
       </c>
       <c r="I81" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J81" t="n">
         <v>2005</v>
       </c>
       <c r="K81" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L81" t="b">
         <v>1</v>
       </c>
       <c r="M81" t="n">
-        <v>16.7192042598665</v>
+        <v>15.7746961170676</v>
       </c>
       <c r="N81" t="n">
-        <v>0.228935884807721</v>
+        <v>0.276558340253779</v>
       </c>
       <c r="O81" t="n">
-        <v>0.00953016845045274</v>
+        <v>0.00103336552605391</v>
       </c>
       <c r="P81" t="s">
         <v>50</v>
@@ -4642,7 +4642,7 @@
         <v>84</v>
       </c>
       <c r="H82" t="n">
-        <v>1206</v>
+        <v>1280</v>
       </c>
       <c r="I82" t="n">
         <v>10</v>
@@ -4657,13 +4657,13 @@
         <v>1</v>
       </c>
       <c r="M82" t="n">
-        <v>65.3698281914598</v>
+        <v>57.578898983305</v>
       </c>
       <c r="N82" t="n">
-        <v>-0.690905530896764</v>
+        <v>-0.376754052299389</v>
       </c>
       <c r="O82" t="n">
-        <v>0.0545337671929453</v>
+        <v>0.295357422338898</v>
       </c>
       <c r="P82" t="s">
         <v>23</v>
@@ -4692,7 +4692,7 @@
         <v>84</v>
       </c>
       <c r="H83" t="n">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="I83" t="n">
         <v>10</v>
@@ -4824,7 +4824,7 @@
         <v>84</v>
       </c>
       <c r="H86" t="n">
-        <v>744</v>
+        <v>799</v>
       </c>
       <c r="I86" t="n">
         <v>10</v>
@@ -4839,13 +4839,13 @@
         <v>1</v>
       </c>
       <c r="M86" t="n">
-        <v>19.5096247739125</v>
+        <v>24.5642568847679</v>
       </c>
       <c r="N86" t="n">
-        <v>1.07987826960051</v>
+        <v>0.873658294447068</v>
       </c>
       <c r="O86" t="n">
-        <v>0.0510252959384295</v>
+        <v>0.141337566141349</v>
       </c>
       <c r="P86" t="s">
         <v>23</v>
@@ -4874,7 +4874,7 @@
         <v>84</v>
       </c>
       <c r="H87" t="n">
-        <v>1481</v>
+        <v>1577</v>
       </c>
       <c r="I87" t="n">
         <v>10</v>
@@ -4889,13 +4889,13 @@
         <v>1</v>
       </c>
       <c r="M87" t="n">
-        <v>88.2665217996213</v>
+        <v>76.7899394419268</v>
       </c>
       <c r="N87" t="n">
-        <v>-1.0880291412905</v>
+        <v>-0.628213299436875</v>
       </c>
       <c r="O87" t="n">
-        <v>0.0665589908704265</v>
+        <v>0.219850271952525</v>
       </c>
       <c r="P87" t="s">
         <v>23</v>
@@ -4924,7 +4924,7 @@
         <v>84</v>
       </c>
       <c r="H88" t="n">
-        <v>1488</v>
+        <v>1584</v>
       </c>
       <c r="I88" t="n">
         <v>10</v>
@@ -4939,13 +4939,13 @@
         <v>1</v>
       </c>
       <c r="M88" t="n">
-        <v>81.4549321940367</v>
+        <v>69.8553875919234</v>
       </c>
       <c r="N88" t="n">
-        <v>-0.870800717005251</v>
+        <v>-0.406426083197994</v>
       </c>
       <c r="O88" t="n">
-        <v>0.162325709325709</v>
+        <v>0.446153345812438</v>
       </c>
       <c r="P88" t="s">
         <v>23</v>
@@ -4989,13 +4989,13 @@
         <v>1</v>
       </c>
       <c r="M89" t="n">
-        <v>-11.3752419427044</v>
+        <v>-11.3750931452145</v>
       </c>
       <c r="N89" t="n">
-        <v>0.911812319697717</v>
+        <v>0.911809230536335</v>
       </c>
       <c r="O89" t="n">
-        <v>0.257183683959014</v>
+        <v>0.257189987451246</v>
       </c>
       <c r="P89" t="s">
         <v>23</v>
@@ -5039,13 +5039,13 @@
         <v>1</v>
       </c>
       <c r="M90" t="n">
-        <v>8.35234095660149</v>
+        <v>8.35281139076768</v>
       </c>
       <c r="N90" t="n">
-        <v>0.370306147987355</v>
+        <v>0.370292305966821</v>
       </c>
       <c r="O90" t="n">
-        <v>0.179767123461435</v>
+        <v>0.179777077709195</v>
       </c>
       <c r="P90" t="s">
         <v>23</v>
@@ -5089,13 +5089,13 @@
         <v>1</v>
       </c>
       <c r="M91" t="n">
-        <v>20.7923996517557</v>
+        <v>20.7923996941562</v>
       </c>
       <c r="N91" t="n">
-        <v>-0.124768398790134</v>
+        <v>-0.124768401354064</v>
       </c>
       <c r="O91" t="n">
-        <v>0.0762040102975333</v>
+        <v>0.0762040357190241</v>
       </c>
       <c r="P91" t="s">
         <v>23</v>
@@ -5226,11 +5226,17 @@
       <c r="L94" t="b">
         <v>1</v>
       </c>
-      <c r="M94"/>
-      <c r="N94"/>
-      <c r="O94"/>
+      <c r="M94" t="n">
+        <v>4.26200141596094</v>
+      </c>
+      <c r="N94" t="n">
+        <v>-0.0392873673000695</v>
+      </c>
+      <c r="O94" t="n">
+        <v>0.79552038130418</v>
+      </c>
       <c r="P94" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
     </row>
     <row r="95">
@@ -5271,13 +5277,13 @@
         <v>1</v>
       </c>
       <c r="M95" t="n">
-        <v>46.71552547721</v>
+        <v>46.7155255141935</v>
       </c>
       <c r="N95" t="n">
-        <v>-0.256647134401874</v>
+        <v>-0.25664713624158</v>
       </c>
       <c r="O95" t="n">
-        <v>0.622020809866009</v>
+        <v>0.622020803450261</v>
       </c>
       <c r="P95" t="s">
         <v>23</v>
@@ -5321,13 +5327,13 @@
         <v>1</v>
       </c>
       <c r="M96" t="n">
-        <v>32.4929157277508</v>
+        <v>32.4933425051872</v>
       </c>
       <c r="N96" t="n">
-        <v>-0.222486917305148</v>
+        <v>-0.222504844024384</v>
       </c>
       <c r="O96" t="n">
-        <v>0.13531248608327</v>
+        <v>0.135218056033289</v>
       </c>
       <c r="P96" t="s">
         <v>23</v>
@@ -5371,13 +5377,13 @@
         <v>1</v>
       </c>
       <c r="M97" t="n">
-        <v>25.2522880735145</v>
+        <v>25.2522887980839</v>
       </c>
       <c r="N97" t="n">
-        <v>-0.198908341061871</v>
+        <v>-0.198908399709913</v>
       </c>
       <c r="O97" t="n">
-        <v>0.00835907721159932</v>
+        <v>0.0083590244169381</v>
       </c>
       <c r="P97" t="s">
         <v>21</v>
@@ -5446,31 +5452,25 @@
         <v>43</v>
       </c>
       <c r="H99" t="n">
-        <v>15696</v>
+        <v>16571</v>
       </c>
       <c r="I99" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J99" t="n">
         <v>1997</v>
       </c>
       <c r="K99" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L99" t="b">
         <v>1</v>
       </c>
-      <c r="M99" t="n">
-        <v>32.8521341427534</v>
-      </c>
-      <c r="N99" t="n">
-        <v>-1.29609511066979</v>
-      </c>
-      <c r="O99" t="n">
-        <v>0.00000000000000000203314969174893</v>
-      </c>
+      <c r="M99"/>
+      <c r="N99"/>
+      <c r="O99"/>
       <c r="P99" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
     </row>
     <row r="100">
@@ -5496,28 +5496,28 @@
         <v>43</v>
       </c>
       <c r="H100" t="n">
-        <v>47168</v>
+        <v>49792</v>
       </c>
       <c r="I100" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J100" t="n">
         <v>1997</v>
       </c>
       <c r="K100" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L100" t="b">
         <v>1</v>
       </c>
       <c r="M100" t="n">
-        <v>0.5326841297858</v>
+        <v>0.486526056048551</v>
       </c>
       <c r="N100" t="n">
-        <v>-0.00517714511339364</v>
+        <v>-0.00182694608070625</v>
       </c>
       <c r="O100" t="n">
-        <v>0.470825738059433</v>
+        <v>0.790980253872378</v>
       </c>
       <c r="P100" t="s">
         <v>23</v>
@@ -5546,28 +5546,28 @@
         <v>43</v>
       </c>
       <c r="H101" t="n">
-        <v>15731</v>
+        <v>16606</v>
       </c>
       <c r="I101" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J101" t="n">
         <v>1997</v>
       </c>
       <c r="K101" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L101" t="b">
         <v>1</v>
       </c>
       <c r="M101" t="n">
-        <v>0.248551179646674</v>
+        <v>0.236691163978561</v>
       </c>
       <c r="N101" t="n">
-        <v>-0.0116683014031875</v>
+        <v>-0.0108992148815637</v>
       </c>
       <c r="O101" t="n">
-        <v>0.102660869939191</v>
+        <v>0.101584432953808</v>
       </c>
       <c r="P101" t="s">
         <v>23</v>
@@ -5596,28 +5596,28 @@
         <v>43</v>
       </c>
       <c r="H102" t="n">
-        <v>15713</v>
+        <v>16588</v>
       </c>
       <c r="I102" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J102" t="n">
         <v>1997</v>
       </c>
       <c r="K102" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L102" t="b">
         <v>1</v>
       </c>
       <c r="M102" t="n">
-        <v>5.71140192386024</v>
+        <v>5.51511737333523</v>
       </c>
       <c r="N102" t="n">
-        <v>-0.240739223450457</v>
+        <v>-0.226783227475027</v>
       </c>
       <c r="O102" t="n">
-        <v>0.00444282141171528</v>
+        <v>0.00433585695109475</v>
       </c>
       <c r="P102" t="s">
         <v>21</v>
@@ -5646,28 +5646,28 @@
         <v>43</v>
       </c>
       <c r="H103" t="n">
-        <v>15732</v>
+        <v>16607</v>
       </c>
       <c r="I103" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J103" t="n">
         <v>1997</v>
       </c>
       <c r="K103" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L103" t="b">
         <v>1</v>
       </c>
       <c r="M103" t="n">
-        <v>1.77734297189416</v>
+        <v>1.73354024142037</v>
       </c>
       <c r="N103" t="n">
-        <v>-0.0692776737501035</v>
+        <v>-0.0663118425822811</v>
       </c>
       <c r="O103" t="n">
-        <v>0.0975863166895465</v>
+        <v>0.0982887196272221</v>
       </c>
       <c r="P103" t="s">
         <v>23</v>
@@ -5696,28 +5696,28 @@
         <v>43</v>
       </c>
       <c r="H104" t="n">
-        <v>16847</v>
+        <v>17779</v>
       </c>
       <c r="I104" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="J104" t="n">
         <v>1994</v>
       </c>
       <c r="K104" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L104" t="b">
         <v>1</v>
       </c>
       <c r="M104" t="n">
-        <v>40.9489597043255</v>
+        <v>39.5068520511913</v>
       </c>
       <c r="N104" t="n">
-        <v>-1.58756424936694</v>
+        <v>-1.47099758677916</v>
       </c>
       <c r="O104" t="n">
-        <v>0.000000000000000000000000375303601367998</v>
+        <v>0.000000000000000000000227816605153144</v>
       </c>
       <c r="P104" t="s">
         <v>21</v>
@@ -5826,28 +5826,28 @@
         <v>43</v>
       </c>
       <c r="H107" t="n">
-        <v>6282</v>
+        <v>6463</v>
       </c>
       <c r="I107" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J107" t="n">
         <v>1998</v>
       </c>
       <c r="K107" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L107" t="b">
         <v>1</v>
       </c>
       <c r="M107" t="n">
-        <v>28.9769326403196</v>
+        <v>27.8792723214916</v>
       </c>
       <c r="N107" t="n">
-        <v>-0.860722448728973</v>
+        <v>-0.781423231347227</v>
       </c>
       <c r="O107" t="n">
-        <v>0.000465450211115611</v>
+        <v>0.000692330268166631</v>
       </c>
       <c r="P107" t="s">
         <v>21</v>
@@ -5876,28 +5876,28 @@
         <v>43</v>
       </c>
       <c r="H108" t="n">
-        <v>18889</v>
+        <v>19432</v>
       </c>
       <c r="I108" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J108" t="n">
         <v>1998</v>
       </c>
       <c r="K108" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L108" t="b">
         <v>1</v>
       </c>
       <c r="M108" t="n">
-        <v>0.0856620604066337</v>
+        <v>0.122749951618511</v>
       </c>
       <c r="N108" t="n">
-        <v>0.0127947855670413</v>
+        <v>0.0100819714820314</v>
       </c>
       <c r="O108" t="n">
-        <v>0.051190785675201</v>
+        <v>0.0940962608088782</v>
       </c>
       <c r="P108" t="s">
         <v>23</v>
@@ -5926,28 +5926,28 @@
         <v>43</v>
       </c>
       <c r="H109" t="n">
-        <v>6301</v>
+        <v>6482</v>
       </c>
       <c r="I109" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J109" t="n">
         <v>1998</v>
       </c>
       <c r="K109" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L109" t="b">
         <v>1</v>
       </c>
       <c r="M109" t="n">
-        <v>0.132184335834842</v>
+        <v>0.12929124115708</v>
       </c>
       <c r="N109" t="n">
-        <v>-0.00512498893664424</v>
+        <v>-0.00491355372019899</v>
       </c>
       <c r="O109" t="n">
-        <v>0.118498663142494</v>
+        <v>0.117004457167443</v>
       </c>
       <c r="P109" t="s">
         <v>23</v>
@@ -5976,28 +5976,28 @@
         <v>43</v>
       </c>
       <c r="H110" t="n">
-        <v>6285</v>
+        <v>6466</v>
       </c>
       <c r="I110" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J110" t="n">
         <v>1998</v>
       </c>
       <c r="K110" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L110" t="b">
         <v>1</v>
       </c>
       <c r="M110" t="n">
-        <v>15.8420696008404</v>
+        <v>15.4835024422216</v>
       </c>
       <c r="N110" t="n">
-        <v>-0.572226245026019</v>
+        <v>-0.545921328667188</v>
       </c>
       <c r="O110" t="n">
-        <v>0.0419864765441194</v>
+        <v>0.0432676395822031</v>
       </c>
       <c r="P110" t="s">
         <v>21</v>
@@ -6026,28 +6026,28 @@
         <v>43</v>
       </c>
       <c r="H111" t="n">
-        <v>6284</v>
+        <v>6465</v>
       </c>
       <c r="I111" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J111" t="n">
         <v>1998</v>
       </c>
       <c r="K111" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L111" t="b">
         <v>1</v>
       </c>
       <c r="M111" t="n">
-        <v>5.71565828377176</v>
+        <v>5.64851568155711</v>
       </c>
       <c r="N111" t="n">
-        <v>-0.196830926179655</v>
+        <v>-0.191974164438094</v>
       </c>
       <c r="O111" t="n">
-        <v>0.0148174763903749</v>
+        <v>0.0143482789438823</v>
       </c>
       <c r="P111" t="s">
         <v>21</v>
@@ -6076,28 +6076,28 @@
         <v>43</v>
       </c>
       <c r="H112" t="n">
-        <v>6815</v>
+        <v>6996</v>
       </c>
       <c r="I112" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="J112" t="n">
         <v>1994</v>
       </c>
       <c r="K112" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L112" t="b">
         <v>1</v>
       </c>
       <c r="M112" t="n">
-        <v>52.3021115018918</v>
+        <v>51.2627695986105</v>
       </c>
       <c r="N112" t="n">
-        <v>-1.69151017812222</v>
+        <v>-1.6030053316693</v>
       </c>
       <c r="O112" t="n">
-        <v>0.0000000000000000000403137535049784</v>
+        <v>0.000000000000000000379808349181876</v>
       </c>
       <c r="P112" t="s">
         <v>21</v>
@@ -6206,31 +6206,31 @@
         <v>90</v>
       </c>
       <c r="H115" t="n">
-        <v>5685</v>
+        <v>6524</v>
       </c>
       <c r="I115" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J115" t="n">
         <v>1997</v>
       </c>
       <c r="K115" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L115" t="b">
         <v>1</v>
       </c>
       <c r="M115" t="n">
-        <v>9.29711141295766</v>
+        <v>8.40851784757194</v>
       </c>
       <c r="N115" t="n">
-        <v>-0.212868634808103</v>
+        <v>-0.148105183067089</v>
       </c>
       <c r="O115" t="n">
-        <v>0.00405168065247469</v>
+        <v>0.0974653898461681</v>
       </c>
       <c r="P115" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="116">
@@ -6256,31 +6256,31 @@
         <v>90</v>
       </c>
       <c r="H116" t="n">
-        <v>17103</v>
+        <v>19627</v>
       </c>
       <c r="I116" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J116" t="n">
         <v>1997</v>
       </c>
       <c r="K116" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L116" t="b">
         <v>1</v>
       </c>
       <c r="M116" t="n">
-        <v>1.70960213659336</v>
+        <v>1.6572921266286</v>
       </c>
       <c r="N116" t="n">
-        <v>-0.0289760355144765</v>
+        <v>-0.0265739062221367</v>
       </c>
       <c r="O116" t="n">
-        <v>0.0448824668545934</v>
+        <v>0.0562321879273083</v>
       </c>
       <c r="P116" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="117">
@@ -6306,16 +6306,16 @@
         <v>43</v>
       </c>
       <c r="H117" t="n">
-        <v>5708</v>
+        <v>6550</v>
       </c>
       <c r="I117" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J117" t="n">
         <v>1997</v>
       </c>
       <c r="K117" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L117" t="b">
         <v>1</v>
@@ -6350,28 +6350,28 @@
         <v>90</v>
       </c>
       <c r="H118" t="n">
-        <v>5698</v>
+        <v>6539</v>
       </c>
       <c r="I118" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J118" t="n">
         <v>1997</v>
       </c>
       <c r="K118" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L118" t="b">
         <v>1</v>
       </c>
       <c r="M118" t="n">
-        <v>17.0121024167292</v>
+        <v>16.2742009880887</v>
       </c>
       <c r="N118" t="n">
-        <v>-0.601666634628676</v>
+        <v>-0.560687169914942</v>
       </c>
       <c r="O118" t="n">
-        <v>0.000235157766530186</v>
+        <v>0.000440849275728977</v>
       </c>
       <c r="P118" t="s">
         <v>21</v>
@@ -6400,28 +6400,28 @@
         <v>90</v>
       </c>
       <c r="H119" t="n">
-        <v>5704</v>
+        <v>6546</v>
       </c>
       <c r="I119" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J119" t="n">
         <v>1997</v>
       </c>
       <c r="K119" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L119" t="b">
         <v>1</v>
       </c>
       <c r="M119" t="n">
-        <v>3.15078674404518</v>
+        <v>3.15642486026929</v>
       </c>
       <c r="N119" t="n">
-        <v>-0.0902733509283717</v>
+        <v>-0.0916237650356675</v>
       </c>
       <c r="O119" t="n">
-        <v>0.0629403377939821</v>
+        <v>0.0657011378680577</v>
       </c>
       <c r="P119" t="s">
         <v>23</v>
@@ -6450,28 +6450,28 @@
         <v>43</v>
       </c>
       <c r="H120" t="n">
-        <v>6231</v>
+        <v>7130</v>
       </c>
       <c r="I120" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="J120" t="n">
         <v>1994</v>
       </c>
       <c r="K120" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L120" t="b">
         <v>1</v>
       </c>
       <c r="M120" t="n">
-        <v>33.1820675646515</v>
+        <v>30.0048298261178</v>
       </c>
       <c r="N120" t="n">
-        <v>-0.932472937767339</v>
+        <v>-0.774268496697167</v>
       </c>
       <c r="O120" t="n">
-        <v>0.000000000909265706738429</v>
+        <v>0.0000155735740157106</v>
       </c>
       <c r="P120" t="s">
         <v>21</v>
@@ -6555,13 +6555,13 @@
         <v>1</v>
       </c>
       <c r="M122" t="n">
-        <v>-1.17225767267301</v>
+        <v>-1.17179361635508</v>
       </c>
       <c r="N122" t="n">
-        <v>0.471000050425961</v>
+        <v>0.470981420692621</v>
       </c>
       <c r="O122" t="n">
-        <v>0.260006328269154</v>
+        <v>0.26003557319771</v>
       </c>
       <c r="P122" t="s">
         <v>23</v>
@@ -6605,13 +6605,13 @@
         <v>1</v>
       </c>
       <c r="M123" t="n">
-        <v>22.5309932608729</v>
+        <v>22.5309932775823</v>
       </c>
       <c r="N123" t="n">
-        <v>-0.54427506679597</v>
+        <v>-0.544275067565711</v>
       </c>
       <c r="O123" t="n">
-        <v>0.0227362276911171</v>
+        <v>0.0227362274662352</v>
       </c>
       <c r="P123" t="s">
         <v>21</v>
@@ -6655,13 +6655,13 @@
         <v>1</v>
       </c>
       <c r="M124" t="n">
-        <v>28.6856935920826</v>
+        <v>28.6857141770335</v>
       </c>
       <c r="N124" t="n">
-        <v>0.18877470936749</v>
+        <v>0.188773694286756</v>
       </c>
       <c r="O124" t="n">
-        <v>0.598317226968351</v>
+        <v>0.598320943514704</v>
       </c>
       <c r="P124" t="s">
         <v>23</v>
@@ -6749,13 +6749,13 @@
         <v>1</v>
       </c>
       <c r="M126" t="n">
-        <v>6.7838230486559</v>
+        <v>6.78381819418626</v>
       </c>
       <c r="N126" t="n">
-        <v>-0.00866126850207299</v>
+        <v>-0.00866100704994314</v>
       </c>
       <c r="O126" t="n">
-        <v>0.962696671246064</v>
+        <v>0.962697808501246</v>
       </c>
       <c r="P126" t="s">
         <v>23</v>
@@ -6799,13 +6799,13 @@
         <v>1</v>
       </c>
       <c r="M127" t="n">
-        <v>4.31520743264204</v>
+        <v>4.31520743264218</v>
       </c>
       <c r="N127" t="n">
-        <v>0.303859009487904</v>
+        <v>0.303859009487899</v>
       </c>
       <c r="O127" t="n">
-        <v>0.453703957656639</v>
+        <v>0.453703957656648</v>
       </c>
       <c r="P127" t="s">
         <v>23</v>
@@ -6849,13 +6849,13 @@
         <v>1</v>
       </c>
       <c r="M128" t="n">
-        <v>26.6419579439412</v>
+        <v>26.6419579439417</v>
       </c>
       <c r="N128" t="n">
-        <v>0.549443451096866</v>
+        <v>0.549443451096848</v>
       </c>
       <c r="O128" t="n">
-        <v>0.246787900026726</v>
+        <v>0.246787900026742</v>
       </c>
       <c r="P128" t="s">
         <v>23</v>
@@ -6884,16 +6884,16 @@
         <v>96</v>
       </c>
       <c r="H129" t="n">
-        <v>102</v>
+        <v>164</v>
       </c>
       <c r="I129" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J129" t="n">
         <v>2024</v>
       </c>
       <c r="K129" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L129" t="b">
         <v>0</v>
@@ -6928,16 +6928,16 @@
         <v>96</v>
       </c>
       <c r="H130" t="n">
-        <v>46</v>
+        <v>74</v>
       </c>
       <c r="I130" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J130" t="n">
         <v>2024</v>
       </c>
       <c r="K130" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L130" t="b">
         <v>0</v>
@@ -6972,16 +6972,16 @@
         <v>96</v>
       </c>
       <c r="H131" t="n">
-        <v>46</v>
+        <v>74</v>
       </c>
       <c r="I131" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J131" t="n">
         <v>2024</v>
       </c>
       <c r="K131" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L131" t="b">
         <v>0</v>
@@ -7016,16 +7016,16 @@
         <v>96</v>
       </c>
       <c r="H132" t="n">
-        <v>46</v>
+        <v>74</v>
       </c>
       <c r="I132" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J132" t="n">
         <v>2024</v>
       </c>
       <c r="K132" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L132" t="b">
         <v>0</v>
@@ -7060,16 +7060,16 @@
         <v>96</v>
       </c>
       <c r="H133" t="n">
-        <v>236</v>
+        <v>386</v>
       </c>
       <c r="I133" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J133" t="n">
         <v>2024</v>
       </c>
       <c r="K133" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L133" t="b">
         <v>0</v>
@@ -7104,16 +7104,16 @@
         <v>96</v>
       </c>
       <c r="H134" t="n">
-        <v>239</v>
+        <v>395</v>
       </c>
       <c r="I134" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J134" t="n">
         <v>2024</v>
       </c>
       <c r="K134" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L134" t="b">
         <v>0</v>
@@ -7188,28 +7188,28 @@
         <v>99</v>
       </c>
       <c r="H136" t="n">
-        <v>787</v>
+        <v>825</v>
       </c>
       <c r="I136" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="J136" t="n">
         <v>1999</v>
       </c>
       <c r="K136" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L136" t="b">
         <v>1</v>
       </c>
       <c r="M136" t="n">
-        <v>20.2590676274871</v>
+        <v>20.19534170184</v>
       </c>
       <c r="N136" t="n">
-        <v>-0.585651209477301</v>
+        <v>-0.580645182704668</v>
       </c>
       <c r="O136" t="n">
-        <v>0.000000000612876949887699</v>
+        <v>0.00000000000192769985029779</v>
       </c>
       <c r="P136" t="s">
         <v>21</v>
@@ -7238,28 +7238,28 @@
         <v>99</v>
       </c>
       <c r="H137" t="n">
-        <v>2379</v>
+        <v>2493</v>
       </c>
       <c r="I137" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="J137" t="n">
         <v>1999</v>
       </c>
       <c r="K137" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L137" t="b">
         <v>1</v>
       </c>
       <c r="M137" t="n">
-        <v>1.73766058924645</v>
+        <v>1.71485988102386</v>
       </c>
       <c r="N137" t="n">
-        <v>-0.0414814042766983</v>
+        <v>-0.0397867824814792</v>
       </c>
       <c r="O137" t="n">
-        <v>0.00089542577025922</v>
+        <v>0.00052505111566868</v>
       </c>
       <c r="P137" t="s">
         <v>21</v>
@@ -7288,16 +7288,16 @@
         <v>43</v>
       </c>
       <c r="H138" t="n">
-        <v>794</v>
+        <v>832</v>
       </c>
       <c r="I138" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="J138" t="n">
         <v>1999</v>
       </c>
       <c r="K138" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L138" t="b">
         <v>1</v>
@@ -7332,28 +7332,28 @@
         <v>99</v>
       </c>
       <c r="H139" t="n">
-        <v>794</v>
+        <v>832</v>
       </c>
       <c r="I139" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="J139" t="n">
         <v>1999</v>
       </c>
       <c r="K139" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L139" t="b">
         <v>1</v>
       </c>
       <c r="M139" t="n">
-        <v>2.54661101365288</v>
+        <v>2.53951567181357</v>
       </c>
       <c r="N139" t="n">
-        <v>-0.0783803494115895</v>
+        <v>-0.0779050940846131</v>
       </c>
       <c r="O139" t="n">
-        <v>0.341034362519376</v>
+        <v>0.336338821176729</v>
       </c>
       <c r="P139" t="s">
         <v>23</v>
@@ -7382,28 +7382,28 @@
         <v>99</v>
       </c>
       <c r="H140" t="n">
-        <v>794</v>
+        <v>832</v>
       </c>
       <c r="I140" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="J140" t="n">
         <v>1999</v>
       </c>
       <c r="K140" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L140" t="b">
         <v>1</v>
       </c>
       <c r="M140" t="n">
-        <v>0.098278249125969</v>
+        <v>0.0937987919740479</v>
       </c>
       <c r="N140" t="n">
-        <v>-0.00433663859300799</v>
+        <v>-0.00400475632155672</v>
       </c>
       <c r="O140" t="n">
-        <v>0.300757978603717</v>
+        <v>0.30074758659337</v>
       </c>
       <c r="P140" t="s">
         <v>23</v>
@@ -7432,28 +7432,28 @@
         <v>43</v>
       </c>
       <c r="H141" t="n">
-        <v>801</v>
+        <v>839</v>
       </c>
       <c r="I141" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="J141" t="n">
         <v>1999</v>
       </c>
       <c r="K141" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L141" t="b">
         <v>1</v>
       </c>
       <c r="M141" t="n">
-        <v>27.7613215210498</v>
+        <v>27.6619615739441</v>
       </c>
       <c r="N141" t="n">
-        <v>-0.805416122805826</v>
+        <v>-0.798741167412668</v>
       </c>
       <c r="O141" t="n">
-        <v>0.000000000000000111937158369317</v>
+        <v>0.00000000000000000216796064709784</v>
       </c>
       <c r="P141" t="s">
         <v>21</v>
@@ -7581,13 +7581,13 @@
         <v>1</v>
       </c>
       <c r="M144" t="n">
-        <v>-5.87122204063504</v>
+        <v>-5.87122250558736</v>
       </c>
       <c r="N144" t="n">
-        <v>1.10079105954384</v>
+        <v>1.10079108471336</v>
       </c>
       <c r="O144" t="n">
-        <v>0.104749045024336</v>
+        <v>0.10474902248809</v>
       </c>
       <c r="P144" t="s">
         <v>23</v>
@@ -7631,13 +7631,13 @@
         <v>1</v>
       </c>
       <c r="M145" t="n">
-        <v>19.6311429839962</v>
+        <v>19.6311429839964</v>
       </c>
       <c r="N145" t="n">
-        <v>0.076522796846791</v>
+        <v>0.076522796846781</v>
       </c>
       <c r="O145" t="n">
-        <v>0.880505716452414</v>
+        <v>0.88050571645243</v>
       </c>
       <c r="P145" t="s">
         <v>23</v>
@@ -7725,13 +7725,13 @@
         <v>1</v>
       </c>
       <c r="M147" t="n">
-        <v>2.64228139828149</v>
+        <v>2.64228139022739</v>
       </c>
       <c r="N147" t="n">
-        <v>0.068164801565837</v>
+        <v>0.0681648019802267</v>
       </c>
       <c r="O147" t="n">
-        <v>0.780887509020257</v>
+        <v>0.780887507542741</v>
       </c>
       <c r="P147" t="s">
         <v>23</v>
@@ -7903,13 +7903,13 @@
         <v>1</v>
       </c>
       <c r="M151" t="n">
-        <v>26.6035655592804</v>
+        <v>26.6035655592142</v>
       </c>
       <c r="N151" t="n">
-        <v>-0.476510204710198</v>
+        <v>-0.476510204712189</v>
       </c>
       <c r="O151" t="n">
-        <v>0.158331973909321</v>
+        <v>0.158331973904867</v>
       </c>
       <c r="P151" t="s">
         <v>23</v>
@@ -7953,13 +7953,13 @@
         <v>1</v>
       </c>
       <c r="M152" t="n">
-        <v>33.4466492799093</v>
+        <v>33.4466492799094</v>
       </c>
       <c r="N152" t="n">
-        <v>-0.526271498290103</v>
+        <v>-0.526271498290106</v>
       </c>
       <c r="O152" t="n">
-        <v>0.134250711812301</v>
+        <v>0.134250711812299</v>
       </c>
       <c r="P152" t="s">
         <v>23</v>
@@ -8072,31 +8072,31 @@
         <v>43</v>
       </c>
       <c r="H155" t="n">
-        <v>651</v>
+        <v>685</v>
       </c>
       <c r="I155" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J155" t="n">
         <v>2009</v>
       </c>
       <c r="K155" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L155" t="b">
         <v>1</v>
       </c>
       <c r="M155" t="n">
-        <v>23.024903019627</v>
+        <v>3.70618582273872</v>
       </c>
       <c r="N155" t="n">
-        <v>-0.773531254197164</v>
+        <v>0.206821431032827</v>
       </c>
       <c r="O155" t="n">
-        <v>0.0202146218231972</v>
+        <v>0.238304224446081</v>
       </c>
       <c r="P155" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="156">
@@ -8122,28 +8122,28 @@
         <v>43</v>
       </c>
       <c r="H156" t="n">
-        <v>1953</v>
+        <v>2055</v>
       </c>
       <c r="I156" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J156" t="n">
         <v>2009</v>
       </c>
       <c r="K156" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L156" t="b">
         <v>1</v>
       </c>
       <c r="M156" t="n">
-        <v>-0.0711150985564275</v>
+        <v>-0.053610494193918</v>
       </c>
       <c r="N156" t="n">
-        <v>0.00372022338125094</v>
+        <v>0.00283405115336671</v>
       </c>
       <c r="O156" t="n">
-        <v>0.167941461820667</v>
+        <v>0.161567647341493</v>
       </c>
       <c r="P156" t="s">
         <v>23</v>
@@ -8172,16 +8172,16 @@
         <v>43</v>
       </c>
       <c r="H157" t="n">
-        <v>651</v>
+        <v>685</v>
       </c>
       <c r="I157" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J157" t="n">
         <v>2009</v>
       </c>
       <c r="K157" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L157" t="b">
         <v>1</v>
@@ -8216,16 +8216,16 @@
         <v>43</v>
       </c>
       <c r="H158" t="n">
-        <v>651</v>
+        <v>685</v>
       </c>
       <c r="I158" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J158" t="n">
         <v>2009</v>
       </c>
       <c r="K158" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L158" t="b">
         <v>1</v>
@@ -8260,16 +8260,16 @@
         <v>43</v>
       </c>
       <c r="H159" t="n">
-        <v>651</v>
+        <v>685</v>
       </c>
       <c r="I159" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J159" t="n">
         <v>2009</v>
       </c>
       <c r="K159" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L159" t="b">
         <v>1</v>
@@ -8304,31 +8304,31 @@
         <v>43</v>
       </c>
       <c r="H160" t="n">
-        <v>651</v>
+        <v>685</v>
       </c>
       <c r="I160" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J160" t="n">
         <v>2009</v>
       </c>
       <c r="K160" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L160" t="b">
         <v>1</v>
       </c>
       <c r="M160" t="n">
-        <v>22.9814232107145</v>
+        <v>3.67438898821875</v>
       </c>
       <c r="N160" t="n">
-        <v>-0.771190976570732</v>
+        <v>0.208564609640469</v>
       </c>
       <c r="O160" t="n">
-        <v>0.0197959930482142</v>
+        <v>0.236718465491046</v>
       </c>
       <c r="P160" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="161">
@@ -8394,31 +8394,31 @@
         <v>52</v>
       </c>
       <c r="H162" t="n">
-        <v>3587</v>
+        <v>4768</v>
       </c>
       <c r="I162" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J162" t="n">
         <v>1997</v>
       </c>
       <c r="K162" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L162" t="b">
         <v>1</v>
       </c>
       <c r="M162" t="n">
-        <v>19.1499706613022</v>
+        <v>18.460796557458</v>
       </c>
       <c r="N162" t="n">
-        <v>-0.316165778379042</v>
+        <v>-0.319419682122757</v>
       </c>
       <c r="O162" t="n">
-        <v>0.0160054813216538</v>
+        <v>0.431503009244388</v>
       </c>
       <c r="P162" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="163">
@@ -8444,31 +8444,31 @@
         <v>52</v>
       </c>
       <c r="H163" t="n">
-        <v>1902</v>
+        <v>2561</v>
       </c>
       <c r="I163" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J163" t="n">
         <v>1997</v>
       </c>
       <c r="K163" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L163" t="b">
         <v>1</v>
       </c>
       <c r="M163" t="n">
-        <v>10.2242875322034</v>
+        <v>14.4442975501166</v>
       </c>
       <c r="N163" t="n">
-        <v>-0.0105453906843651</v>
+        <v>-0.166055290313739</v>
       </c>
       <c r="O163" t="n">
-        <v>0.870075455176696</v>
+        <v>0.038264187108685</v>
       </c>
       <c r="P163" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="164">
@@ -8494,28 +8494,28 @@
         <v>52</v>
       </c>
       <c r="H164" t="n">
-        <v>540</v>
+        <v>678</v>
       </c>
       <c r="I164" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="J164" t="n">
         <v>1997</v>
       </c>
       <c r="K164" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L164" t="b">
         <v>1</v>
       </c>
       <c r="M164" t="n">
-        <v>8.34583588573481</v>
+        <v>8.7879312105827</v>
       </c>
       <c r="N164" t="n">
-        <v>0.122351783460449</v>
+        <v>0.0927755833398184</v>
       </c>
       <c r="O164" t="n">
-        <v>0.294839445823322</v>
+        <v>0.38946976613155</v>
       </c>
       <c r="P164" t="s">
         <v>23</v>
@@ -8544,16 +8544,16 @@
         <v>52</v>
       </c>
       <c r="H165" t="n">
-        <v>87</v>
+        <v>153</v>
       </c>
       <c r="I165" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J165" t="n">
         <v>1998</v>
       </c>
       <c r="K165" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L165" t="b">
         <v>1</v>
@@ -8588,28 +8588,28 @@
         <v>52</v>
       </c>
       <c r="H166" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="I166" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J166" t="n">
         <v>1997</v>
       </c>
       <c r="K166" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L166" t="b">
         <v>1</v>
       </c>
       <c r="M166" t="n">
-        <v>-9.22516513824099</v>
+        <v>8.39152299448192</v>
       </c>
       <c r="N166" t="n">
-        <v>0.704825482924538</v>
+        <v>0.0442851066408185</v>
       </c>
       <c r="O166" t="n">
-        <v>0.746731107226386</v>
+        <v>0.969004325922695</v>
       </c>
       <c r="P166" t="s">
         <v>23</v>
@@ -8638,28 +8638,28 @@
         <v>52</v>
       </c>
       <c r="H167" t="n">
-        <v>2334</v>
+        <v>2664</v>
       </c>
       <c r="I167" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J167" t="n">
         <v>1997</v>
       </c>
       <c r="K167" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L167" t="b">
         <v>1</v>
       </c>
       <c r="M167" t="n">
-        <v>44.0732080683524</v>
+        <v>57.5162188256729</v>
       </c>
       <c r="N167" t="n">
-        <v>-1.05225252508132</v>
+        <v>-1.51153810685005</v>
       </c>
       <c r="O167" t="n">
-        <v>0.0095643740255073</v>
+        <v>0.00489236123899467</v>
       </c>
       <c r="P167" t="s">
         <v>21</v>
@@ -8688,28 +8688,28 @@
         <v>52</v>
       </c>
       <c r="H168" t="n">
-        <v>7480</v>
+        <v>9473</v>
       </c>
       <c r="I168" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J168" t="n">
         <v>1997</v>
       </c>
       <c r="K168" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L168" t="b">
         <v>1</v>
       </c>
       <c r="M168" t="n">
-        <v>108.013733201528</v>
+        <v>113.703116368091</v>
       </c>
       <c r="N168" t="n">
-        <v>-2.56973970312599</v>
+        <v>-2.76905746455337</v>
       </c>
       <c r="O168" t="n">
-        <v>0.00000000008376340262188</v>
+        <v>0.00000000000000480637576416575</v>
       </c>
       <c r="P168" t="s">
         <v>21</v>
@@ -8753,13 +8753,13 @@
         <v>1</v>
       </c>
       <c r="M169" t="n">
-        <v>18.4858461622144</v>
+        <v>18.4858461593842</v>
       </c>
       <c r="N169" t="n">
-        <v>-0.57107692313935</v>
+        <v>-0.57107692311824</v>
       </c>
       <c r="O169" t="n">
-        <v>0.0671357481774192</v>
+        <v>0.0671357480917357</v>
       </c>
       <c r="P169" t="s">
         <v>23</v>
@@ -8803,13 +8803,13 @@
         <v>1</v>
       </c>
       <c r="M170" t="n">
-        <v>12.12575641794</v>
+        <v>12.1257564173751</v>
       </c>
       <c r="N170" t="n">
-        <v>-0.0149842466920076</v>
+        <v>-0.0149842466671144</v>
       </c>
       <c r="O170" t="n">
-        <v>0.931856627545226</v>
+        <v>0.931856627659933</v>
       </c>
       <c r="P170" t="s">
         <v>23</v>
@@ -8853,13 +8853,13 @@
         <v>1</v>
       </c>
       <c r="M171" t="n">
-        <v>15.4432607125131</v>
+        <v>15.443260712513</v>
       </c>
       <c r="N171" t="n">
-        <v>0.430165149041331</v>
+        <v>0.430165149041334</v>
       </c>
       <c r="O171" t="n">
-        <v>0.219275347947408</v>
+        <v>0.219275347947406</v>
       </c>
       <c r="P171" t="s">
         <v>23</v>
@@ -9075,13 +9075,13 @@
         <v>1</v>
       </c>
       <c r="M176" t="n">
-        <v>20.588524859885</v>
+        <v>20.5885250687694</v>
       </c>
       <c r="N176" t="n">
-        <v>0.366270848891099</v>
+        <v>0.366270859299474</v>
       </c>
       <c r="O176" t="n">
-        <v>0.283296634236128</v>
+        <v>0.283296617342563</v>
       </c>
       <c r="P176" t="s">
         <v>23</v>
@@ -9125,13 +9125,13 @@
         <v>1</v>
       </c>
       <c r="M177" t="n">
-        <v>8.90779448258092</v>
+        <v>8.90778952009263</v>
       </c>
       <c r="N177" t="n">
-        <v>0.106397105863102</v>
+        <v>0.10639731584783</v>
       </c>
       <c r="O177" t="n">
-        <v>0.459517983463199</v>
+        <v>0.459517067678269</v>
       </c>
       <c r="P177" t="s">
         <v>23</v>
@@ -9175,13 +9175,13 @@
         <v>1</v>
       </c>
       <c r="M178" t="n">
-        <v>19.2737433657372</v>
+        <v>19.2737433657373</v>
       </c>
       <c r="N178" t="n">
-        <v>0.298326138204907</v>
+        <v>0.298326138204902</v>
       </c>
       <c r="O178" t="n">
-        <v>0.328421016947517</v>
+        <v>0.328421016947526</v>
       </c>
       <c r="P178" t="s">
         <v>23</v>
@@ -9225,13 +9225,13 @@
         <v>1</v>
       </c>
       <c r="M179" t="n">
-        <v>1.3465451752785</v>
+        <v>1.34638775200742</v>
       </c>
       <c r="N179" t="n">
-        <v>-0.0087296070060331</v>
+        <v>-0.00872276598730886</v>
       </c>
       <c r="O179" t="n">
-        <v>0.956323793332353</v>
+        <v>0.956357577347309</v>
       </c>
       <c r="P179" t="s">
         <v>23</v>
@@ -9260,28 +9260,28 @@
         <v>110</v>
       </c>
       <c r="H180" t="n">
-        <v>1022</v>
+        <v>1086</v>
       </c>
       <c r="I180" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J180" t="n">
         <v>2012</v>
       </c>
       <c r="K180" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L180" t="b">
         <v>1</v>
       </c>
       <c r="M180" t="n">
-        <v>-49.5920796655998</v>
+        <v>-49.761290412474</v>
       </c>
       <c r="N180" t="n">
-        <v>2.66186726637865</v>
+        <v>2.67373427225315</v>
       </c>
       <c r="O180" t="n">
-        <v>0.00000239090453057941</v>
+        <v>0.00000318809996200969</v>
       </c>
       <c r="P180" t="s">
         <v>50</v>
@@ -9310,28 +9310,28 @@
         <v>110</v>
       </c>
       <c r="H181" t="n">
-        <v>7113</v>
+        <v>7125</v>
       </c>
       <c r="I181" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J181" t="n">
         <v>1998</v>
       </c>
       <c r="K181" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L181" t="b">
         <v>1</v>
       </c>
       <c r="M181" t="n">
-        <v>23.4170769887968</v>
+        <v>23.582597929326</v>
       </c>
       <c r="N181" t="n">
-        <v>0.214241051756911</v>
+        <v>0.205904459580598</v>
       </c>
       <c r="O181" t="n">
-        <v>0.129962039390411</v>
+        <v>0.145713233948874</v>
       </c>
       <c r="P181" t="s">
         <v>23</v>
@@ -9404,16 +9404,16 @@
         <v>112</v>
       </c>
       <c r="H183" t="n">
-        <v>3935</v>
+        <v>3961</v>
       </c>
       <c r="I183" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J183" t="n">
         <v>1998</v>
       </c>
       <c r="K183" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L183" t="b">
         <v>1</v>
@@ -9463,13 +9463,13 @@
         <v>1</v>
       </c>
       <c r="M184" t="n">
-        <v>-20.7185464749576</v>
+        <v>-20.7179114764626</v>
       </c>
       <c r="N184" t="n">
-        <v>1.16038099050171</v>
+        <v>1.16034761795276</v>
       </c>
       <c r="O184" t="n">
-        <v>0.368350598684456</v>
+        <v>0.368359158553326</v>
       </c>
       <c r="P184" t="s">
         <v>23</v>
@@ -9498,28 +9498,28 @@
         <v>110</v>
       </c>
       <c r="H185" t="n">
-        <v>4590</v>
+        <v>4621</v>
       </c>
       <c r="I185" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J185" t="n">
         <v>1998</v>
       </c>
       <c r="K185" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L185" t="b">
         <v>1</v>
       </c>
       <c r="M185" t="n">
-        <v>19.3045368009947</v>
+        <v>19.9314858536334</v>
       </c>
       <c r="N185" t="n">
-        <v>0.357128673128779</v>
+        <v>0.326801795878895</v>
       </c>
       <c r="O185" t="n">
-        <v>0.078279096280564</v>
+        <v>0.114315322088279</v>
       </c>
       <c r="P185" t="s">
         <v>23</v>
@@ -9548,28 +9548,28 @@
         <v>110</v>
       </c>
       <c r="H186" t="n">
-        <v>4025</v>
+        <v>4071</v>
       </c>
       <c r="I186" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J186" t="n">
         <v>1998</v>
       </c>
       <c r="K186" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L186" t="b">
         <v>1</v>
       </c>
       <c r="M186" t="n">
-        <v>41.8688979916643</v>
+        <v>42.2151159553225</v>
       </c>
       <c r="N186" t="n">
-        <v>-0.195129154789458</v>
+        <v>-0.212197716071814</v>
       </c>
       <c r="O186" t="n">
-        <v>0.232466977105312</v>
+        <v>0.196587032046407</v>
       </c>
       <c r="P186" t="s">
         <v>23</v>
@@ -9613,13 +9613,13 @@
         <v>1</v>
       </c>
       <c r="M187" t="n">
-        <v>35.6054197123911</v>
+        <v>35.6054215170507</v>
       </c>
       <c r="N187" t="n">
-        <v>0.419915563194657</v>
+        <v>0.419915469481326</v>
       </c>
       <c r="O187" t="n">
-        <v>0.574127622659356</v>
+        <v>0.574127834383349</v>
       </c>
       <c r="P187" t="s">
         <v>23</v>
@@ -9663,13 +9663,13 @@
         <v>1</v>
       </c>
       <c r="M188" t="n">
-        <v>-1.6366623620019</v>
+        <v>-1.63664205039697</v>
       </c>
       <c r="N188" t="n">
-        <v>0.109313418689803</v>
+        <v>0.109312346931521</v>
       </c>
       <c r="O188" t="n">
-        <v>0.658163700860897</v>
+        <v>0.658167263124645</v>
       </c>
       <c r="P188" t="s">
         <v>23</v>
@@ -9713,13 +9713,13 @@
         <v>1</v>
       </c>
       <c r="M189" t="n">
-        <v>33.628723773395</v>
+        <v>33.6286656016465</v>
       </c>
       <c r="N189" t="n">
-        <v>-1.70910436858776</v>
+        <v>-1.70909816755082</v>
       </c>
       <c r="O189" t="n">
-        <v>0.254590618263364</v>
+        <v>0.254605077074609</v>
       </c>
       <c r="P189" t="s">
         <v>23</v>
@@ -9763,13 +9763,13 @@
         <v>1</v>
       </c>
       <c r="M190" t="n">
-        <v>-0.44456113092958</v>
+        <v>-0.444567344856501</v>
       </c>
       <c r="N190" t="n">
-        <v>0.0784241882663684</v>
+        <v>0.0784251979579704</v>
       </c>
       <c r="O190" t="n">
-        <v>0.356281826344633</v>
+        <v>0.356262072866792</v>
       </c>
       <c r="P190" t="s">
         <v>23</v>
@@ -9813,13 +9813,13 @@
         <v>1</v>
       </c>
       <c r="M191" t="n">
-        <v>3.53048070193436</v>
+        <v>3.53048514537169</v>
       </c>
       <c r="N191" t="n">
-        <v>-0.232326898201871</v>
+        <v>-0.23232673623941</v>
       </c>
       <c r="O191" t="n">
-        <v>0.44371379125858</v>
+        <v>0.443711658627369</v>
       </c>
       <c r="P191" t="s">
         <v>23</v>
@@ -9863,13 +9863,13 @@
         <v>1</v>
       </c>
       <c r="M192" t="n">
-        <v>16.1048036953012</v>
+        <v>16.1047804901159</v>
       </c>
       <c r="N192" t="n">
-        <v>-1.13438778746813</v>
+        <v>-1.13438365908922</v>
       </c>
       <c r="O192" t="n">
-        <v>0.40008285596946</v>
+        <v>0.400085578534954</v>
       </c>
       <c r="P192" t="s">
         <v>23</v>
@@ -9913,13 +9913,13 @@
         <v>1</v>
       </c>
       <c r="M193" t="n">
-        <v>36.9900137332185</v>
+        <v>36.9900159752838</v>
       </c>
       <c r="N193" t="n">
-        <v>-3.13814583526341</v>
+        <v>-3.13814594958305</v>
       </c>
       <c r="O193" t="n">
-        <v>0.0666608562339737</v>
+        <v>0.0666593236207905</v>
       </c>
       <c r="P193" t="s">
         <v>23</v>
@@ -9963,13 +9963,13 @@
         <v>1</v>
       </c>
       <c r="M194" t="n">
-        <v>68.369484917475</v>
+        <v>68.3692745038019</v>
       </c>
       <c r="N194" t="n">
-        <v>-4.52097026315786</v>
+        <v>-4.52094347983225</v>
       </c>
       <c r="O194" t="n">
-        <v>0.0166182622893285</v>
+        <v>0.0166190751416014</v>
       </c>
       <c r="P194" t="s">
         <v>21</v>
@@ -10013,13 +10013,13 @@
         <v>1</v>
       </c>
       <c r="M195" t="n">
-        <v>33.6286514164965</v>
+        <v>33.6286656016465</v>
       </c>
       <c r="N195" t="n">
-        <v>-1.70909712972767</v>
+        <v>-1.70909816755082</v>
       </c>
       <c r="O195" t="n">
-        <v>0.254620455536205</v>
+        <v>0.254605077074609</v>
       </c>
       <c r="P195" t="s">
         <v>23</v>
@@ -10063,13 +10063,13 @@
         <v>1</v>
       </c>
       <c r="M196" t="n">
-        <v>-0.444559760659897</v>
+        <v>-0.444567344856501</v>
       </c>
       <c r="N196" t="n">
-        <v>0.0784239357792856</v>
+        <v>0.0784251979579704</v>
       </c>
       <c r="O196" t="n">
-        <v>0.356289780424534</v>
+        <v>0.356262072866792</v>
       </c>
       <c r="P196" t="s">
         <v>23</v>
@@ -10113,13 +10113,13 @@
         <v>1</v>
       </c>
       <c r="M197" t="n">
-        <v>3.53048964166756</v>
+        <v>3.53048514537169</v>
       </c>
       <c r="N197" t="n">
-        <v>-0.232327351261614</v>
+        <v>-0.23232673623941</v>
       </c>
       <c r="O197" t="n">
-        <v>0.443714818400394</v>
+        <v>0.443711658627369</v>
       </c>
       <c r="P197" t="s">
         <v>23</v>
@@ -10163,13 +10163,13 @@
         <v>1</v>
       </c>
       <c r="M198" t="n">
-        <v>16.104786187905</v>
+        <v>16.1047804901159</v>
       </c>
       <c r="N198" t="n">
-        <v>-1.13438480926907</v>
+        <v>-1.13438365908922</v>
       </c>
       <c r="O198" t="n">
-        <v>0.400089904762928</v>
+        <v>0.400085578534954</v>
       </c>
       <c r="P198" t="s">
         <v>23</v>
@@ -10213,13 +10213,13 @@
         <v>1</v>
       </c>
       <c r="M199" t="n">
-        <v>36.9899401290369</v>
+        <v>36.9900159752838</v>
       </c>
       <c r="N199" t="n">
-        <v>-3.13813606811501</v>
+        <v>-3.13814594958305</v>
       </c>
       <c r="O199" t="n">
-        <v>0.0666627263574941</v>
+        <v>0.0666593236207905</v>
       </c>
       <c r="P199" t="s">
         <v>23</v>
@@ -10263,13 +10263,13 @@
         <v>1</v>
       </c>
       <c r="M200" t="n">
-        <v>68.3694284976308</v>
+        <v>68.3692745038019</v>
       </c>
       <c r="N200" t="n">
-        <v>-4.52096298854313</v>
+        <v>-4.52094347983225</v>
       </c>
       <c r="O200" t="n">
-        <v>0.0166183943820369</v>
+        <v>0.0166190751416014</v>
       </c>
       <c r="P200" t="s">
         <v>21</v>
@@ -10313,13 +10313,13 @@
         <v>1</v>
       </c>
       <c r="M201" t="n">
-        <v>84.4240519069693</v>
+        <v>84.4240521172969</v>
       </c>
       <c r="N201" t="n">
-        <v>-2.62425690745865</v>
+        <v>-2.62425691537163</v>
       </c>
       <c r="O201" t="n">
-        <v>0.0740357829782734</v>
+        <v>0.0740357853759614</v>
       </c>
       <c r="P201" t="s">
         <v>23</v>
@@ -10363,13 +10363,13 @@
         <v>1</v>
       </c>
       <c r="M202" t="n">
-        <v>11.9869803982023</v>
+        <v>11.986980400469</v>
       </c>
       <c r="N202" t="n">
-        <v>0.27052871967714</v>
+        <v>0.27052871960507</v>
       </c>
       <c r="O202" t="n">
-        <v>0.485492239784015</v>
+        <v>0.485492239666146</v>
       </c>
       <c r="P202" t="s">
         <v>23</v>
@@ -10457,13 +10457,13 @@
         <v>1</v>
       </c>
       <c r="M204" t="n">
-        <v>4.17278690398094</v>
+        <v>4.17278654215605</v>
       </c>
       <c r="N204" t="n">
-        <v>-0.151389667982695</v>
+        <v>-0.15138953086087</v>
       </c>
       <c r="O204" t="n">
-        <v>0.819593974777737</v>
+        <v>0.819593916025816</v>
       </c>
       <c r="P204" t="s">
         <v>23</v>
@@ -10507,13 +10507,13 @@
         <v>1</v>
       </c>
       <c r="M205" t="n">
-        <v>27.0389698918424</v>
+        <v>27.0389687993447</v>
       </c>
       <c r="N205" t="n">
-        <v>1.06249137834728</v>
+        <v>1.06249142248844</v>
       </c>
       <c r="O205" t="n">
-        <v>0.131535963264703</v>
+        <v>0.131535964561105</v>
       </c>
       <c r="P205" t="s">
         <v>23</v>
@@ -10557,13 +10557,13 @@
         <v>1</v>
       </c>
       <c r="M206" t="n">
-        <v>88.1358699273268</v>
+        <v>88.1362868491369</v>
       </c>
       <c r="N206" t="n">
-        <v>-1.52267574045742</v>
+        <v>-1.52272482880892</v>
       </c>
       <c r="O206" t="n">
-        <v>0.15021973127204</v>
+        <v>0.150214626938448</v>
       </c>
       <c r="P206" t="s">
         <v>23</v>
@@ -10607,13 +10607,13 @@
         <v>1</v>
       </c>
       <c r="M207" t="n">
-        <v>9.61203743636063</v>
+        <v>9.61203742621614</v>
       </c>
       <c r="N207" t="n">
-        <v>0.0838012513185918</v>
+        <v>0.0838012516893737</v>
       </c>
       <c r="O207" t="n">
-        <v>0.831389754186489</v>
+        <v>0.831389753629501</v>
       </c>
       <c r="P207" t="s">
         <v>23</v>
@@ -10657,13 +10657,13 @@
         <v>1</v>
       </c>
       <c r="M208" t="n">
-        <v>48.4483227974256</v>
+        <v>48.4483227947062</v>
       </c>
       <c r="N208" t="n">
-        <v>-0.491452101443074</v>
+        <v>-0.491452101326007</v>
       </c>
       <c r="O208" t="n">
-        <v>0.503221346965114</v>
+        <v>0.503221347188028</v>
       </c>
       <c r="P208" t="s">
         <v>23</v>
@@ -10751,13 +10751,13 @@
         <v>1</v>
       </c>
       <c r="M210" t="n">
-        <v>54.1977529427332</v>
+        <v>54.1971703449698</v>
       </c>
       <c r="N210" t="n">
-        <v>-0.898615908276998</v>
+        <v>-0.898587802225779</v>
       </c>
       <c r="O210" t="n">
-        <v>0.25668244223902</v>
+        <v>0.256698903785388</v>
       </c>
       <c r="P210" t="s">
         <v>23</v>
@@ -10801,13 +10801,13 @@
         <v>1</v>
       </c>
       <c r="M211" t="n">
-        <v>62.380384729702</v>
+        <v>62.3803683883504</v>
       </c>
       <c r="N211" t="n">
-        <v>-0.142093645741606</v>
+        <v>-0.142093117878052</v>
       </c>
       <c r="O211" t="n">
-        <v>0.687476149885152</v>
+        <v>0.687476157247382</v>
       </c>
       <c r="P211" t="s">
         <v>23</v>
@@ -10836,28 +10836,28 @@
         <v>52</v>
       </c>
       <c r="H212" t="n">
-        <v>1200</v>
+        <v>1328</v>
       </c>
       <c r="I212" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J212" t="n">
         <v>1997</v>
       </c>
       <c r="K212" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L212" t="b">
         <v>1</v>
       </c>
       <c r="M212" t="n">
-        <v>17.6001377016579</v>
+        <v>18.4230481020772</v>
       </c>
       <c r="N212" t="n">
-        <v>-0.177242116605302</v>
+        <v>-0.224003186251882</v>
       </c>
       <c r="O212" t="n">
-        <v>0.214505464474497</v>
+        <v>0.103428972363119</v>
       </c>
       <c r="P212" t="s">
         <v>23</v>
@@ -10886,28 +10886,28 @@
         <v>52</v>
       </c>
       <c r="H213" t="n">
-        <v>1488</v>
+        <v>1631</v>
       </c>
       <c r="I213" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J213" t="n">
         <v>1997</v>
       </c>
       <c r="K213" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L213" t="b">
         <v>1</v>
       </c>
       <c r="M213" t="n">
-        <v>24.3152173700395</v>
+        <v>27.1359792559161</v>
       </c>
       <c r="N213" t="n">
-        <v>-0.107824398497227</v>
+        <v>-0.261424059195711</v>
       </c>
       <c r="O213" t="n">
-        <v>0.554386983760942</v>
+        <v>0.1437116811893</v>
       </c>
       <c r="P213" t="s">
         <v>23</v>
@@ -10936,31 +10936,31 @@
         <v>52</v>
       </c>
       <c r="H214" t="n">
-        <v>468</v>
+        <v>503</v>
       </c>
       <c r="I214" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="J214" t="n">
         <v>1997</v>
       </c>
       <c r="K214" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L214" t="b">
         <v>1</v>
       </c>
       <c r="M214" t="n">
-        <v>63.8891206981744</v>
+        <v>75.1431686053921</v>
       </c>
       <c r="N214" t="n">
-        <v>-1.75638883870463</v>
+        <v>-2.16214489044141</v>
       </c>
       <c r="O214" t="n">
-        <v>0.0916263907051741</v>
+        <v>0.044702954339368</v>
       </c>
       <c r="P214" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="215">
@@ -10986,16 +10986,16 @@
         <v>52</v>
       </c>
       <c r="H215" t="n">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="I215" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J215" t="n">
         <v>1997</v>
       </c>
       <c r="K215" t="n">
-        <v>2021</v>
+        <v>2025</v>
       </c>
       <c r="L215" t="b">
         <v>1</v>
@@ -11030,28 +11030,28 @@
         <v>52</v>
       </c>
       <c r="H216" t="n">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="I216" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J216" t="n">
         <v>1997</v>
       </c>
       <c r="K216" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L216" t="b">
         <v>1</v>
       </c>
       <c r="M216" t="n">
-        <v>23.3867558483777</v>
+        <v>23.5414554090611</v>
       </c>
       <c r="N216" t="n">
-        <v>-0.134009146040018</v>
+        <v>-0.163019815792196</v>
       </c>
       <c r="O216" t="n">
-        <v>0.724458235015615</v>
+        <v>0.664093711204479</v>
       </c>
       <c r="P216" t="s">
         <v>23</v>
@@ -11080,28 +11080,28 @@
         <v>52</v>
       </c>
       <c r="H217" t="n">
-        <v>722</v>
+        <v>747</v>
       </c>
       <c r="I217" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J217" t="n">
         <v>1997</v>
       </c>
       <c r="K217" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L217" t="b">
         <v>1</v>
       </c>
       <c r="M217" t="n">
-        <v>17.2241548079113</v>
+        <v>18.494359011557</v>
       </c>
       <c r="N217" t="n">
-        <v>-0.0625766221763471</v>
+        <v>-0.134124424203036</v>
       </c>
       <c r="O217" t="n">
-        <v>0.744519670631815</v>
+        <v>0.511251330606643</v>
       </c>
       <c r="P217" t="s">
         <v>23</v>
@@ -11130,28 +11130,28 @@
         <v>52</v>
       </c>
       <c r="H218" t="n">
-        <v>3169</v>
+        <v>3260</v>
       </c>
       <c r="I218" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J218" t="n">
         <v>1997</v>
       </c>
       <c r="K218" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L218" t="b">
         <v>1</v>
       </c>
       <c r="M218" t="n">
-        <v>34.9835958039344</v>
+        <v>36.1626677265256</v>
       </c>
       <c r="N218" t="n">
-        <v>-0.111791462313524</v>
+        <v>-0.183596335695938</v>
       </c>
       <c r="O218" t="n">
-        <v>0.468477051061486</v>
+        <v>0.249088171024273</v>
       </c>
       <c r="P218" t="s">
         <v>23</v>
@@ -11239,13 +11239,13 @@
         <v>1</v>
       </c>
       <c r="M220" t="n">
-        <v>25.7351476699093</v>
+        <v>25.7351476699092</v>
       </c>
       <c r="N220" t="n">
-        <v>0.862848997722571</v>
+        <v>0.862848997722573</v>
       </c>
       <c r="O220" t="n">
-        <v>0.0041757479179363</v>
+        <v>0.00417574791793629</v>
       </c>
       <c r="P220" t="s">
         <v>50</v>
@@ -11380,10 +11380,10 @@
         <v>36.5374750333897</v>
       </c>
       <c r="N223" t="n">
-        <v>0.141924957308237</v>
+        <v>0.141924957308238</v>
       </c>
       <c r="O223" t="n">
-        <v>0.708114476390104</v>
+        <v>0.708114476390101</v>
       </c>
       <c r="P223" t="s">
         <v>23</v>
@@ -11427,13 +11427,13 @@
         <v>1</v>
       </c>
       <c r="M224" t="n">
-        <v>34.4313177493422</v>
+        <v>34.4313177493427</v>
       </c>
       <c r="N224" t="n">
-        <v>0.22966300140264</v>
+        <v>0.229663001402628</v>
       </c>
       <c r="O224" t="n">
-        <v>0.446908276330284</v>
+        <v>0.446908276330308</v>
       </c>
       <c r="P224" t="s">
         <v>23</v>

</xml_diff>